<commit_message>
feat: added unit tests (2 of 2), finished testing phase
</commit_message>
<xml_diff>
--- a/Tests/Integrated Tests/integrated_tests.xlsx
+++ b/Tests/Integrated Tests/integrated_tests.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mortrpestl\Desktop\Archives\mortrpestl\The UPper Hand\1st Year\1st Sem\CS11\cs11project\cs11-project-jugemu-jugemu\Tests\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mortrpestl\Desktop\Archives\mortrpestl\The UPper Hand\1st Year\1st Sem\CS11\cs11project\cs11-project-jugemu-jugemu\Tests\Integrated Tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD6558C0-5ADC-43A7-A2ED-8781F9910064}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A3A8AA2-04A0-4F18-93A2-F9A216A60A99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="473" uniqueCount="341">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="472" uniqueCount="341">
   <si>
     <t>Unnamed: 0</t>
   </si>
@@ -3898,7 +3898,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -4205,7 +4205,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H79"/>
+  <dimension ref="A1:H78"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="9.06640625" style="5"/>
@@ -6097,11 +6097,6 @@
         <v>45962</v>
       </c>
     </row>
-    <row r="79" spans="1:8" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A79" s="2" t="s">
-        <v>333</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
fix: edited reset logic
</commit_message>
<xml_diff>
--- a/Tests/Integrated Tests/integrated_tests.xlsx
+++ b/Tests/Integrated Tests/integrated_tests.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mortrpestl\Desktop\Archives\mortrpestl\The UPper Hand\1st Year\1st Sem\CS11\cs11project\cs11-project-jugemu-jugemu\Tests\Integrated Tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A3A8AA2-04A0-4F18-93A2-F9A216A60A99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E1CC34A-5F43-4EE4-B2B7-1E5444DDDA47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="472" uniqueCount="341">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="472" uniqueCount="340">
   <si>
     <t>Unnamed: 0</t>
   </si>
@@ -3596,22 +3596,7 @@
     <t>71</t>
   </si>
   <si>
-    <t>Attempt to move after reset in the same string</t>
-  </si>
-  <si>
     <t>ww!aaaaaaaaaaa</t>
-  </si>
-  <si>
-    <t>NO CLEAR
-TTTTTTTTTTTTTTTTTTTT
-T..................T
-T..................T
-T.....~....+.+.....T
-T.....~......+.....T
-T.....~............T
-T..........L.......T
-T..................T
-TTTTTTTTTTTTTTTTTTTT</t>
   </si>
   <si>
     <t>72</t>
@@ -3817,6 +3802,9 @@
 T........T
 T......~.T
 TTTTTTTTTT</t>
+  </si>
+  <si>
+    <t>Attempt to move after reset in the same string (should still run)</t>
   </si>
 </sst>
 </file>
@@ -4240,7 +4228,7 @@
         <v>6</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="156.75" x14ac:dyDescent="0.45">
@@ -4257,7 +4245,7 @@
         <v>10</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>12</v>
@@ -5427,7 +5415,7 @@
         <v>218</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="D51" s="2" t="s">
         <v>219</v>
@@ -5939,16 +5927,16 @@
         <v>307</v>
       </c>
       <c r="C72" s="2" t="s">
-        <v>308</v>
+        <v>339</v>
       </c>
       <c r="D72" s="2" t="s">
         <v>292</v>
       </c>
       <c r="E72" s="2" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="F72" s="2" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="G72" s="2"/>
       <c r="H72" s="4">
@@ -5960,19 +5948,19 @@
         <v>254</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="C73" s="2" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="D73" s="2" t="s">
         <v>292</v>
       </c>
       <c r="E73" s="2" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="F73" s="2" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="G73" s="2"/>
       <c r="H73" s="4">
@@ -5981,22 +5969,22 @@
     </row>
     <row r="74" spans="1:8" ht="156.75" x14ac:dyDescent="0.45">
       <c r="A74" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="B74" s="2" t="s">
+        <v>314</v>
+      </c>
+      <c r="C74" s="2" t="s">
         <v>315</v>
       </c>
-      <c r="B74" s="2" t="s">
+      <c r="D74" s="2" t="s">
         <v>316</v>
       </c>
-      <c r="C74" s="2" t="s">
+      <c r="E74" s="2" t="s">
         <v>317</v>
       </c>
-      <c r="D74" s="2" t="s">
+      <c r="F74" s="2" t="s">
         <v>318</v>
-      </c>
-      <c r="E74" s="2" t="s">
-        <v>319</v>
-      </c>
-      <c r="F74" s="2" t="s">
-        <v>320</v>
       </c>
       <c r="G74" s="2"/>
       <c r="H74" s="4">
@@ -6005,22 +5993,22 @@
     </row>
     <row r="75" spans="1:8" ht="156.75" x14ac:dyDescent="0.45">
       <c r="A75" s="2" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="B75" s="2" t="s">
+        <v>319</v>
+      </c>
+      <c r="C75" s="2" t="s">
+        <v>320</v>
+      </c>
+      <c r="D75" s="2" t="s">
+        <v>316</v>
+      </c>
+      <c r="E75" s="2" t="s">
         <v>321</v>
       </c>
-      <c r="C75" s="2" t="s">
+      <c r="F75" s="2" t="s">
         <v>322</v>
-      </c>
-      <c r="D75" s="2" t="s">
-        <v>318</v>
-      </c>
-      <c r="E75" s="2" t="s">
-        <v>323</v>
-      </c>
-      <c r="F75" s="2" t="s">
-        <v>324</v>
       </c>
       <c r="G75" s="2"/>
       <c r="H75" s="4">
@@ -6029,22 +6017,22 @@
     </row>
     <row r="76" spans="1:8" ht="409.5" x14ac:dyDescent="0.45">
       <c r="A76" s="2" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="B76" s="2" t="s">
+        <v>323</v>
+      </c>
+      <c r="C76" s="2" t="s">
+        <v>324</v>
+      </c>
+      <c r="D76" s="2" t="s">
         <v>325</v>
       </c>
-      <c r="C76" s="2" t="s">
+      <c r="E76" s="2" t="s">
         <v>326</v>
       </c>
-      <c r="D76" s="2" t="s">
+      <c r="F76" s="2" t="s">
         <v>327</v>
-      </c>
-      <c r="E76" s="2" t="s">
-        <v>328</v>
-      </c>
-      <c r="F76" s="2" t="s">
-        <v>329</v>
       </c>
       <c r="G76" s="2"/>
       <c r="H76" s="4">
@@ -6053,22 +6041,22 @@
     </row>
     <row r="77" spans="1:8" ht="85.5" x14ac:dyDescent="0.45">
       <c r="A77" s="2" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="B77" s="5">
         <v>76</v>
       </c>
       <c r="C77" s="2" t="s">
+        <v>332</v>
+      </c>
+      <c r="D77" s="2" t="s">
         <v>334</v>
       </c>
-      <c r="D77" s="2" t="s">
+      <c r="E77" s="5" t="s">
         <v>336</v>
       </c>
-      <c r="E77" s="5" t="s">
-        <v>338</v>
-      </c>
       <c r="F77" s="2" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="H77" s="4">
         <v>45962</v>
@@ -6076,22 +6064,22 @@
     </row>
     <row r="78" spans="1:8" ht="85.5" x14ac:dyDescent="0.45">
       <c r="A78" s="2" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="B78" s="5">
         <v>77</v>
       </c>
       <c r="C78" s="2" t="s">
+        <v>333</v>
+      </c>
+      <c r="D78" s="2" t="s">
+        <v>334</v>
+      </c>
+      <c r="E78" s="5" t="s">
         <v>335</v>
       </c>
-      <c r="D78" s="2" t="s">
-        <v>336</v>
-      </c>
-      <c r="E78" s="5" t="s">
-        <v>337</v>
-      </c>
       <c r="F78" s="2" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="H78" s="4">
         <v>45962</v>

</xml_diff>